<commit_message>
cambios despues de correccion
</commit_message>
<xml_diff>
--- a/outputs/anexo13_calculado_con_tus_datos.xlsx
+++ b/outputs/anexo13_calculado_con_tus_datos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Muestra_1_t_pareada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Muestra_2_one_sample_t" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Muestra_1_t_pareada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Muestra_2_one_sample_t" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,17 +418,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>pre</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>post</t>
         </is>
@@ -453,10 +441,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.86734693877551</v>
+        <v>2.846938775510204</v>
       </c>
       <c r="C2" t="n">
-        <v>5.122448979591836</v>
+        <v>4.469387755102041</v>
       </c>
     </row>
     <row r="3">
@@ -466,10 +454,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.310518053375196</v>
+        <v>1.832862375719519</v>
       </c>
       <c r="C3" t="n">
-        <v>1.646467817896389</v>
+        <v>1.634955520669806</v>
       </c>
     </row>
     <row r="4">
@@ -492,7 +480,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.402760213485606</v>
+        <v>0.4534929865294036</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
@@ -525,7 +513,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-2.312163093471554</v>
+        <v>-16.48844117675165</v>
       </c>
       <c r="C8" t="inlineStr"/>
     </row>
@@ -536,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.01090642851520016</v>
+        <v>4.009339354485901e-39</v>
       </c>
       <c r="C9" t="inlineStr"/>
     </row>
@@ -547,7 +535,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.652705309770755</v>
+        <v>1.652705309771445</v>
       </c>
       <c r="C10" t="inlineStr"/>
     </row>
@@ -558,7 +546,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02181285703040032</v>
+        <v>8.018678708971803e-39</v>
       </c>
       <c r="C11" t="inlineStr"/>
     </row>
@@ -569,7 +557,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.972204051265833</v>
+        <v>1.972204051268443</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
@@ -588,67 +576,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Obs</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Mean</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Std. Err.</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Std. Dev.</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>[95% Conf. Interval] Low</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>[95% Conf. Interval] High</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>t</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>degrees of freedom</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>H0: mean =</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Pr(T &lt; t)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Pr(|T| &gt; |t|)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Pr(T &gt; t)</t>
         </is>
@@ -664,22 +652,22 @@
         <v>196</v>
       </c>
       <c r="C2" t="n">
-        <v>5.122448979591836</v>
+        <v>4.469387755102041</v>
       </c>
       <c r="D2" t="n">
-        <v>0.09165340151721295</v>
+        <v>0.09133241373869272</v>
       </c>
       <c r="E2" t="n">
-        <v>1.283147621240981</v>
+        <v>1.278653792341698</v>
       </c>
       <c r="F2" t="n">
-        <v>4.941689769807295</v>
+        <v>4.289261598714465</v>
       </c>
       <c r="G2" t="n">
-        <v>5.303208189376377</v>
+        <v>4.649513911489616</v>
       </c>
       <c r="H2" t="n">
-        <v>-675.1255272155639</v>
+        <v>-684.6486333296921</v>
       </c>
       <c r="I2" t="n">
         <v>195</v>

</xml_diff>